<commit_message>
Normalize priorities across all 1361 cases; sort filters A-Z; add Excel export
- Priority review (rubric: P1 core/auth/security/data/payment, P2 validation/
  concurrency/negatives, P3 rare/cosmetic): 201 cases re-prioritized
- Update xlsx Priority column for 147 changed API (all) cases
- Sort all filter dropdowns alphabetically (localeCompare vi)
- Add 'Xuat Excel' (.xls) export alongside CSV; both include Steps column

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/API_QC_Test_Case_Template_542_Cases.xlsx
+++ b/API_QC_Test_Case_Template_542_Cases.xlsx
@@ -667,7 +667,7 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1477,7 +1477,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -2001,7 +2001,7 @@
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
@@ -2055,7 +2055,7 @@
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="I35" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J35" s="5" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J68" s="5" t="inlineStr">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="I82" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
       <c r="I83" s="5" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J83" s="5" t="inlineStr">
@@ -10205,7 +10205,7 @@
       </c>
       <c r="I182" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J182" s="5" t="inlineStr">
@@ -10259,7 +10259,7 @@
       </c>
       <c r="I183" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J183" s="5" t="inlineStr">
@@ -10317,7 +10317,7 @@
       </c>
       <c r="I184" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J184" s="5" t="inlineStr">
@@ -10425,7 +10425,7 @@
       </c>
       <c r="I186" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J186" s="5" t="inlineStr">
@@ -10483,7 +10483,7 @@
       </c>
       <c r="I187" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J187" s="5" t="inlineStr">
@@ -10537,7 +10537,7 @@
       </c>
       <c r="I188" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J188" s="5" t="inlineStr">
@@ -10591,7 +10591,7 @@
       </c>
       <c r="I189" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J189" s="5" t="inlineStr">
@@ -10645,7 +10645,7 @@
       </c>
       <c r="I190" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J190" s="5" t="inlineStr">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="I191" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J191" s="5" t="inlineStr">
@@ -10745,7 +10745,7 @@
       </c>
       <c r="I192" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J192" s="5" t="inlineStr">
@@ -10799,7 +10799,7 @@
       </c>
       <c r="I193" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J193" s="5" t="inlineStr">
@@ -10853,7 +10853,7 @@
       </c>
       <c r="I194" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J194" s="5" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="I195" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J195" s="5" t="inlineStr">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="I196" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J196" s="5" t="inlineStr">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="I197" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J197" s="5" t="inlineStr">
@@ -11061,7 +11061,7 @@
       </c>
       <c r="I198" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J198" s="5" t="inlineStr">
@@ -11115,7 +11115,7 @@
       </c>
       <c r="I199" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J199" s="5" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="I215" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J215" s="5" t="inlineStr">
@@ -12025,7 +12025,7 @@
       </c>
       <c r="I216" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J216" s="5" t="inlineStr">
@@ -12075,7 +12075,7 @@
       </c>
       <c r="I217" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J217" s="5" t="inlineStr">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="I218" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J218" s="5" t="inlineStr">
@@ -12183,7 +12183,7 @@
       </c>
       <c r="I219" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J219" s="5" t="inlineStr">
@@ -12283,7 +12283,7 @@
       </c>
       <c r="I221" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J221" s="5" t="inlineStr">
@@ -12333,7 +12333,7 @@
       </c>
       <c r="I222" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J222" s="5" t="inlineStr">
@@ -12383,7 +12383,7 @@
       </c>
       <c r="I223" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J223" s="5" t="inlineStr">
@@ -12433,7 +12433,7 @@
       </c>
       <c r="I224" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J224" s="5" t="inlineStr">
@@ -12487,7 +12487,7 @@
       </c>
       <c r="I225" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J225" s="5" t="inlineStr">
@@ -12537,7 +12537,7 @@
       </c>
       <c r="I226" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J226" s="5" t="inlineStr">
@@ -12591,7 +12591,7 @@
       </c>
       <c r="I227" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J227" s="5" t="inlineStr">
@@ -12641,7 +12641,7 @@
       </c>
       <c r="I228" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J228" s="5" t="inlineStr">
@@ -12799,7 +12799,7 @@
       </c>
       <c r="I231" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J231" s="5" t="inlineStr">
@@ -12853,7 +12853,7 @@
       </c>
       <c r="I232" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J232" s="5" t="inlineStr">
@@ -13585,7 +13585,7 @@
       </c>
       <c r="I246" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J246" s="5" t="inlineStr">
@@ -13635,7 +13635,7 @@
       </c>
       <c r="I247" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J247" s="5" t="inlineStr">
@@ -13685,7 +13685,7 @@
       </c>
       <c r="I248" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J248" s="5" t="inlineStr">
@@ -17493,7 +17493,7 @@
       </c>
       <c r="I320" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J320" s="5" t="inlineStr">
@@ -17551,7 +17551,7 @@
       </c>
       <c r="I321" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J321" s="5" t="inlineStr">
@@ -17609,7 +17609,7 @@
       </c>
       <c r="I322" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J322" s="5" t="inlineStr">
@@ -17667,7 +17667,7 @@
       </c>
       <c r="I323" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J323" s="5" t="inlineStr">
@@ -17725,7 +17725,7 @@
       </c>
       <c r="I324" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J324" s="5" t="inlineStr">
@@ -17783,7 +17783,7 @@
       </c>
       <c r="I325" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J325" s="5" t="inlineStr">
@@ -17841,7 +17841,7 @@
       </c>
       <c r="I326" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J326" s="5" t="inlineStr">
@@ -17899,7 +17899,7 @@
       </c>
       <c r="I327" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J327" s="5" t="inlineStr">
@@ -17957,7 +17957,7 @@
       </c>
       <c r="I328" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J328" s="5" t="inlineStr">
@@ -18015,7 +18015,7 @@
       </c>
       <c r="I329" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J329" s="5" t="inlineStr">
@@ -18065,7 +18065,7 @@
       </c>
       <c r="I330" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J330" s="5" t="inlineStr">
@@ -18115,7 +18115,7 @@
       </c>
       <c r="I331" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J331" s="5" t="inlineStr">
@@ -18165,7 +18165,7 @@
       </c>
       <c r="I332" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J332" s="5" t="inlineStr">
@@ -18215,7 +18215,7 @@
       </c>
       <c r="I333" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J333" s="5" t="inlineStr">
@@ -18265,7 +18265,7 @@
       </c>
       <c r="I334" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J334" s="5" t="inlineStr">
@@ -18315,7 +18315,7 @@
       </c>
       <c r="I335" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J335" s="5" t="inlineStr">
@@ -19667,7 +19667,7 @@
       </c>
       <c r="I361" s="5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J361" s="5" t="inlineStr">
@@ -20629,7 +20629,7 @@
       </c>
       <c r="I380" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J380" s="5" t="inlineStr">
@@ -20679,7 +20679,7 @@
       </c>
       <c r="I381" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J381" s="5" t="inlineStr">
@@ -20729,7 +20729,7 @@
       </c>
       <c r="I382" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J382" s="5" t="inlineStr">
@@ -20779,7 +20779,7 @@
       </c>
       <c r="I383" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J383" s="5" t="inlineStr">
@@ -20829,7 +20829,7 @@
       </c>
       <c r="I384" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J384" s="5" t="inlineStr">
@@ -20879,7 +20879,7 @@
       </c>
       <c r="I385" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J385" s="5" t="inlineStr">
@@ -20929,7 +20929,7 @@
       </c>
       <c r="I386" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J386" s="5" t="inlineStr">
@@ -20979,7 +20979,7 @@
       </c>
       <c r="I387" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J387" s="5" t="inlineStr">
@@ -21033,7 +21033,7 @@
       </c>
       <c r="I388" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J388" s="5" t="inlineStr">
@@ -21087,7 +21087,7 @@
       </c>
       <c r="I389" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J389" s="5" t="inlineStr">
@@ -21141,7 +21141,7 @@
       </c>
       <c r="I390" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J390" s="5" t="inlineStr">
@@ -21191,7 +21191,7 @@
       </c>
       <c r="I391" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J391" s="5" t="inlineStr">
@@ -21241,7 +21241,7 @@
       </c>
       <c r="I392" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J392" s="5" t="inlineStr">
@@ -21291,7 +21291,7 @@
       </c>
       <c r="I393" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J393" s="5" t="inlineStr">
@@ -21341,7 +21341,7 @@
       </c>
       <c r="I394" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J394" s="5" t="inlineStr">
@@ -21391,7 +21391,7 @@
       </c>
       <c r="I395" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J395" s="5" t="inlineStr">
@@ -21441,7 +21441,7 @@
       </c>
       <c r="I396" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J396" s="5" t="inlineStr">
@@ -21491,7 +21491,7 @@
       </c>
       <c r="I397" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J397" s="5" t="inlineStr">
@@ -21541,7 +21541,7 @@
       </c>
       <c r="I398" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J398" s="5" t="inlineStr">
@@ -21591,7 +21591,7 @@
       </c>
       <c r="I399" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J399" s="5" t="inlineStr">
@@ -21641,7 +21641,7 @@
       </c>
       <c r="I400" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J400" s="5" t="inlineStr">
@@ -21691,7 +21691,7 @@
       </c>
       <c r="I401" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J401" s="5" t="inlineStr">
@@ -21799,7 +21799,7 @@
       </c>
       <c r="I403" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J403" s="5" t="inlineStr">
@@ -21849,7 +21849,7 @@
       </c>
       <c r="I404" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J404" s="5" t="inlineStr">
@@ -21899,7 +21899,7 @@
       </c>
       <c r="I405" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J405" s="5" t="inlineStr">
@@ -21949,7 +21949,7 @@
       </c>
       <c r="I406" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J406" s="5" t="inlineStr">
@@ -22003,7 +22003,7 @@
       </c>
       <c r="I407" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J407" s="5" t="inlineStr">
@@ -22053,7 +22053,7 @@
       </c>
       <c r="I408" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J408" s="5" t="inlineStr">
@@ -22103,7 +22103,7 @@
       </c>
       <c r="I409" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J409" s="5" t="inlineStr">
@@ -22153,7 +22153,7 @@
       </c>
       <c r="I410" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J410" s="5" t="inlineStr">
@@ -22203,7 +22203,7 @@
       </c>
       <c r="I411" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J411" s="5" t="inlineStr">
@@ -22253,7 +22253,7 @@
       </c>
       <c r="I412" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J412" s="5" t="inlineStr">
@@ -23165,7 +23165,7 @@
       </c>
       <c r="I430" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J430" s="5" t="inlineStr">
@@ -23215,7 +23215,7 @@
       </c>
       <c r="I431" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J431" s="5" t="inlineStr">
@@ -23265,7 +23265,7 @@
       </c>
       <c r="I432" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J432" s="5" t="inlineStr">
@@ -23315,7 +23315,7 @@
       </c>
       <c r="I433" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J433" s="5" t="inlineStr">
@@ -23365,7 +23365,7 @@
       </c>
       <c r="I434" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J434" s="5" t="inlineStr">
@@ -23415,7 +23415,7 @@
       </c>
       <c r="I435" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J435" s="5" t="inlineStr">
@@ -23465,7 +23465,7 @@
       </c>
       <c r="I436" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J436" s="5" t="inlineStr">
@@ -23515,7 +23515,7 @@
       </c>
       <c r="I437" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J437" s="5" t="inlineStr">
@@ -23565,7 +23565,7 @@
       </c>
       <c r="I438" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J438" s="5" t="inlineStr">
@@ -23623,7 +23623,7 @@
       </c>
       <c r="I439" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J439" s="5" t="inlineStr">
@@ -23673,7 +23673,7 @@
       </c>
       <c r="I440" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J440" s="5" t="inlineStr">
@@ -23723,7 +23723,7 @@
       </c>
       <c r="I441" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J441" s="5" t="inlineStr">
@@ -24023,7 +24023,7 @@
       </c>
       <c r="I447" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J447" s="5" t="inlineStr">
@@ -24073,7 +24073,7 @@
       </c>
       <c r="I448" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J448" s="5" t="inlineStr">
@@ -24123,7 +24123,7 @@
       </c>
       <c r="I449" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="J449" s="5" t="inlineStr">
@@ -24489,7 +24489,7 @@
       </c>
       <c r="I456" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J456" s="5" t="inlineStr">
@@ -24543,7 +24543,7 @@
       </c>
       <c r="I457" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J457" s="5" t="inlineStr">
@@ -25845,7 +25845,7 @@
       </c>
       <c r="I482" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J482" s="5" t="inlineStr">
@@ -25899,7 +25899,7 @@
       </c>
       <c r="I483" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J483" s="5" t="inlineStr">
@@ -25957,7 +25957,7 @@
       </c>
       <c r="I484" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J484" s="5" t="inlineStr">
@@ -26011,7 +26011,7 @@
       </c>
       <c r="I485" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J485" s="5" t="inlineStr">
@@ -26061,7 +26061,7 @@
       </c>
       <c r="I486" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J486" s="5" t="inlineStr">
@@ -26161,7 +26161,7 @@
       </c>
       <c r="I488" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J488" s="5" t="inlineStr">
@@ -28693,7 +28693,7 @@
       </c>
       <c r="I536" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J536" s="5" t="inlineStr">
@@ -28743,7 +28743,7 @@
       </c>
       <c r="I537" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J537" s="5" t="inlineStr">
@@ -28793,7 +28793,7 @@
       </c>
       <c r="I538" s="5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J538" s="5" t="inlineStr">
@@ -28843,7 +28843,7 @@
       </c>
       <c r="I539" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J539" s="5" t="inlineStr">
@@ -28893,7 +28893,7 @@
       </c>
       <c r="I540" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J540" s="5" t="inlineStr">
@@ -28943,7 +28943,7 @@
       </c>
       <c r="I541" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J541" s="5" t="inlineStr">
@@ -28993,7 +28993,7 @@
       </c>
       <c r="I542" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J542" s="5" t="inlineStr">
@@ -29043,7 +29043,7 @@
       </c>
       <c r="I543" s="5" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="J543" s="5" t="inlineStr">

</xml_diff>